<commit_message>
modified script and data
</commit_message>
<xml_diff>
--- a/Supplementary_Material/Parameter_Values.xlsx
+++ b/Supplementary_Material/Parameter_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uibes-my.sharepoint.com/personal/swa020_id_uib_eu/Documents/SAINATH_POST_DOC/OTSun/PTC_Gaussian/Scientific_Reports/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uibes-my.sharepoint.com/personal/swa020_id_uib_eu/Documents/gaussian_backup/Gaussian_Lib/Supplementary_Material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="935" documentId="8_{51F0730E-0DEB-48A6-920F-CCC5CA4F9F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAB58EF5-AEF6-42D2-A7F6-CB7CB454F311}"/>
+  <xr:revisionPtr revIDLastSave="1233" documentId="8_{51F0730E-0DEB-48A6-920F-CCC5CA4F9F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0DE5780-5E0D-42B6-9954-2F51EED09489}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{469DDB95-EBE9-4ED4-83C6-5065F84F5F0B}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="15480" xr2:uid="{469DDB95-EBE9-4ED4-83C6-5065F84F5F0B}"/>
   </bookViews>
   <sheets>
     <sheet name="Jeter" sheetId="7" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Receiver_Diameter" sheetId="2" r:id="rId4"/>
     <sheet name="Receiver_Height" sheetId="1" r:id="rId5"/>
     <sheet name="Rim_Angle" sheetId="3" r:id="rId6"/>
+    <sheet name="Receiver_Diameter _Theta=1" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="83">
   <si>
     <t>A</t>
   </si>
@@ -519,9 +520,6 @@
     <t>Inv. G. [12.5°-77.5°]</t>
   </si>
   <si>
-    <t>Skw. G. [77.5°-1780°]</t>
-  </si>
-  <si>
     <t>Inv. G. [12.5°-72.5°]</t>
   </si>
   <si>
@@ -540,9 +538,6 @@
     <t>GMM4  [0°-180°]</t>
   </si>
   <si>
-    <t>DoG. [0°-12.5°]</t>
-  </si>
-  <si>
     <t>GMM4  [13.5°-180°]</t>
   </si>
   <si>
@@ -561,20 +556,76 @@
     <t>DoG. [0°-13.5°]</t>
   </si>
   <si>
-    <t>Simple G  [0°-180°]</t>
-  </si>
-  <si>
     <t>DoG. [0°-15°]</t>
   </si>
   <si>
     <t>S.M. Jeter 1986, Incidence angle (Degree)</t>
+  </si>
+  <si>
+    <t>DoG. [0°-17.5°]</t>
+  </si>
+  <si>
+    <t>GMM4  [27.5°-180°]</t>
+  </si>
+  <si>
+    <t>Skw. G. [77.5°-180°]</t>
+  </si>
+  <si>
+    <t>GMM4  [-180° to 97.5°]</t>
+  </si>
+  <si>
+    <t>GMM3  [-180° to 97.5°]</t>
+  </si>
+  <si>
+    <t>GMM4  [-180° to 92.5°]</t>
+  </si>
+  <si>
+    <t>GMM4  [-180° to -37.5°]</t>
+  </si>
+  <si>
+    <t>GMM4  [-37.5° to 180°]</t>
+  </si>
+  <si>
+    <t>GMM4  [-180° to -32.5°]</t>
+  </si>
+  <si>
+    <t>GMM4  [-32.5° to 180°]</t>
+  </si>
+  <si>
+    <t>GMM4  [-180° to -30.5°]</t>
+  </si>
+  <si>
+    <t>GMM4  [-30.5° to 180°]</t>
+  </si>
+  <si>
+    <t>Gaussian [97.5° to 180°]</t>
+  </si>
+  <si>
+    <t>Gaussian [92.5° to 180°]</t>
+  </si>
+  <si>
+    <r>
+      <t>Effect of incidence angle, θ =1° and ф = 90</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>°</t>
+    </r>
+  </si>
+  <si>
+    <t>Gaussian  [0°-180°]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -647,6 +698,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -656,7 +719,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -828,11 +891,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -890,6 +962,30 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -898,15 +994,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -919,15 +1006,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -944,10 +1022,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1267,16 +1341,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{409CB138-7E4C-4C0C-9073-96660C3CC360}">
-  <dimension ref="A2:K30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:K29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.21875" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="46.8" x14ac:dyDescent="0.45">
-      <c r="A2" s="36" t="s">
-        <v>69</v>
+    <row r="2" spans="1:11" ht="47.25" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
+        <v>66</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>11</v>
@@ -1309,18 +1383,18 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="29">
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="28">
         <v>0</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>60</v>
+      <c r="B3" s="28" t="s">
+        <v>67</v>
       </c>
       <c r="C3" s="2">
         <v>-973.14</v>
       </c>
       <c r="D3" s="2">
-        <v>80.3</v>
+        <v>8.0299999999999994</v>
       </c>
       <c r="E3" s="2">
         <v>8.48</v>
@@ -1332,11 +1406,11 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="35"/>
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="29"/>
       <c r="B4" s="30"/>
       <c r="C4" s="2">
-        <v>1000.5</v>
+        <v>1001</v>
       </c>
       <c r="D4" s="2">
         <v>8.06</v>
@@ -1351,19 +1425,19 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="35"/>
-      <c r="B5" s="28" t="s">
-        <v>47</v>
+    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="29"/>
+      <c r="B5" s="32" t="s">
+        <v>16</v>
       </c>
       <c r="C5" s="2">
-        <v>34</v>
+        <v>33.31</v>
       </c>
       <c r="D5" s="2">
-        <v>29.7</v>
+        <v>26.58</v>
       </c>
       <c r="E5" s="2">
-        <v>41.62</v>
+        <v>26.67</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1372,17 +1446,17 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="35"/>
-      <c r="B6" s="28"/>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="29"/>
+      <c r="B6" s="32"/>
       <c r="C6" s="2">
-        <v>26.5</v>
+        <v>38.33</v>
       </c>
       <c r="D6" s="2">
-        <v>71.45</v>
+        <v>71.8</v>
       </c>
       <c r="E6" s="2">
-        <v>15.53</v>
+        <v>17.489999999999998</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -1391,17 +1465,17 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="35"/>
-      <c r="B7" s="28"/>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="29"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="2">
-        <v>4.3499999999999996</v>
+        <v>1.02</v>
       </c>
       <c r="D7" s="2">
-        <v>113.36</v>
+        <v>165.04</v>
       </c>
       <c r="E7" s="2">
-        <v>9.01</v>
+        <v>17.59</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1410,17 +1484,21 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="30"/>
-      <c r="B8" s="28"/>
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="28">
+        <v>15</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>64</v>
+      </c>
       <c r="C8" s="2">
-        <v>0.77</v>
+        <v>-974.5</v>
       </c>
       <c r="D8" s="2">
-        <v>170.96</v>
+        <v>8.0299999999999994</v>
       </c>
       <c r="E8" s="2">
-        <v>11.88</v>
+        <v>8.48</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -1429,21 +1507,17 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="29">
-        <v>15</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>66</v>
-      </c>
+    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="29"/>
+      <c r="B9" s="30"/>
       <c r="C9" s="2">
-        <v>-974.5</v>
+        <v>1000.8</v>
       </c>
       <c r="D9" s="2">
-        <v>8.0299999999999994</v>
+        <v>8.06</v>
       </c>
       <c r="E9" s="2">
-        <v>8.48</v>
+        <v>8.67</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1452,17 +1526,19 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="35"/>
-      <c r="B10" s="30"/>
+    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="29"/>
+      <c r="B10" s="28" t="s">
+        <v>59</v>
+      </c>
       <c r="C10" s="2">
-        <v>1000.8</v>
+        <v>35.35</v>
       </c>
       <c r="D10" s="2">
-        <v>8.06</v>
+        <v>54.12</v>
       </c>
       <c r="E10" s="2">
-        <v>8.67</v>
+        <v>73.09</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -1471,19 +1547,17 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="35"/>
-      <c r="B11" s="29" t="s">
-        <v>61</v>
-      </c>
+    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="29"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="2">
-        <v>35.35</v>
+        <v>10.72</v>
       </c>
       <c r="D11" s="2">
-        <v>54.12</v>
+        <v>64.59</v>
       </c>
       <c r="E11" s="2">
-        <v>73.09</v>
+        <v>10.6</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1492,17 +1566,17 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="35"/>
-      <c r="B12" s="35"/>
+    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="29"/>
+      <c r="B12" s="29"/>
       <c r="C12" s="2">
-        <v>10.72</v>
+        <v>14.94</v>
       </c>
       <c r="D12" s="2">
-        <v>64.59</v>
+        <v>110.2</v>
       </c>
       <c r="E12" s="2">
-        <v>10.6</v>
+        <v>15.52</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -1511,17 +1585,17 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="35"/>
-      <c r="B13" s="35"/>
+    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="30"/>
+      <c r="B13" s="30"/>
       <c r="C13" s="2">
-        <v>14.94</v>
+        <v>14.18</v>
       </c>
       <c r="D13" s="2">
-        <v>110.2</v>
+        <v>141.94999999999999</v>
       </c>
       <c r="E13" s="2">
-        <v>15.52</v>
+        <v>29.87</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -1530,63 +1604,63 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="30"/>
-      <c r="B14" s="30"/>
+    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="28">
+        <v>30</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="C14" s="2">
-        <v>14.18</v>
+        <v>4</v>
       </c>
       <c r="D14" s="2">
-        <v>141.94999999999999</v>
+        <v>18.5</v>
       </c>
       <c r="E14" s="2">
-        <v>29.87</v>
+        <v>3.61</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="29">
-        <v>30</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>45</v>
+      <c r="K14" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="29"/>
+      <c r="B15" s="32" t="s">
+        <v>47</v>
       </c>
       <c r="C15" s="2">
-        <v>4</v>
+        <v>26.85</v>
       </c>
       <c r="D15" s="2">
-        <v>18.5</v>
+        <v>20.3</v>
       </c>
       <c r="E15" s="2">
-        <v>3.61</v>
+        <v>31.48</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" s="2">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="35"/>
-      <c r="B16" s="28" t="s">
-        <v>47</v>
-      </c>
+      <c r="K15" s="2"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="29"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="2">
-        <v>26.85</v>
+        <v>28.32</v>
       </c>
       <c r="D16" s="2">
-        <v>20.3</v>
+        <v>70.62</v>
       </c>
       <c r="E16" s="2">
-        <v>31.48</v>
+        <v>20.86</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -1595,17 +1669,17 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="35"/>
-      <c r="B17" s="28"/>
+    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="29"/>
+      <c r="B17" s="32"/>
       <c r="C17" s="2">
-        <v>28.32</v>
+        <v>3.08</v>
       </c>
       <c r="D17" s="2">
-        <v>70.62</v>
+        <v>61.37</v>
       </c>
       <c r="E17" s="2">
-        <v>20.86</v>
+        <v>5.89</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -1614,17 +1688,17 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="35"/>
-      <c r="B18" s="28"/>
+    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="30"/>
+      <c r="B18" s="32"/>
       <c r="C18" s="2">
-        <v>3.08</v>
+        <v>1.31</v>
       </c>
       <c r="D18" s="2">
-        <v>61.37</v>
+        <v>163.09</v>
       </c>
       <c r="E18" s="2">
-        <v>5.89</v>
+        <v>16.53</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -1633,63 +1707,63 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="30"/>
-      <c r="B19" s="28"/>
+    <row r="19" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="28">
+        <v>45</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="C19" s="2">
-        <v>1.31</v>
+        <v>2.8</v>
       </c>
       <c r="D19" s="2">
-        <v>163.09</v>
+        <v>22.5</v>
       </c>
       <c r="E19" s="2">
-        <v>16.53</v>
+        <v>4.78</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-    </row>
-    <row r="20" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="29">
-        <v>45</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>62</v>
+      <c r="K19" s="2">
+        <v>23.2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="29"/>
+      <c r="B20" s="32" t="s">
+        <v>61</v>
       </c>
       <c r="C20" s="2">
-        <v>2.8</v>
+        <v>5.2</v>
       </c>
       <c r="D20" s="2">
-        <v>22.5</v>
+        <v>59.13</v>
       </c>
       <c r="E20" s="2">
-        <v>4.78</v>
+        <v>11.32</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
-      <c r="K20" s="2">
-        <v>23.2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="35"/>
-      <c r="B21" s="28" t="s">
-        <v>63</v>
-      </c>
+      <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="29"/>
+      <c r="B21" s="32"/>
       <c r="C21" s="2">
-        <v>5.2</v>
+        <v>30.39</v>
       </c>
       <c r="D21" s="2">
-        <v>59.13</v>
+        <v>103.71</v>
       </c>
       <c r="E21" s="2">
-        <v>11.32</v>
+        <v>110.87</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1698,17 +1772,17 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="35"/>
-      <c r="B22" s="28"/>
+    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="29"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="2">
-        <v>30.39</v>
+        <v>-16.36</v>
       </c>
       <c r="D22" s="2">
-        <v>103.71</v>
+        <v>113.68</v>
       </c>
       <c r="E22" s="2">
-        <v>110.87</v>
+        <v>23.79</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -1717,17 +1791,17 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="35"/>
-      <c r="B23" s="28"/>
+    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="30"/>
+      <c r="B23" s="32"/>
       <c r="C23" s="2">
-        <v>-16.36</v>
+        <v>-24.2</v>
       </c>
       <c r="D23" s="2">
-        <v>113.68</v>
+        <v>166.71</v>
       </c>
       <c r="E23" s="2">
-        <v>23.79</v>
+        <v>40.200000000000003</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -1736,63 +1810,63 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="30"/>
-      <c r="B24" s="28"/>
+    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="28">
+        <v>60</v>
+      </c>
+      <c r="B24" s="24" t="s">
+        <v>62</v>
+      </c>
       <c r="C24" s="2">
-        <v>-24.2</v>
+        <v>1.52</v>
       </c>
       <c r="D24" s="2">
-        <v>166.71</v>
+        <v>24</v>
       </c>
       <c r="E24" s="2">
-        <v>40.200000000000003</v>
+        <v>4.58</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-    </row>
-    <row r="25" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="29">
-        <v>60</v>
-      </c>
-      <c r="B25" s="24" t="s">
-        <v>64</v>
+      <c r="K24" s="2">
+        <v>17.059999999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="29"/>
+      <c r="B25" s="28" t="s">
+        <v>63</v>
       </c>
       <c r="C25" s="2">
-        <v>1.52</v>
+        <v>-2.78</v>
       </c>
       <c r="D25" s="2">
-        <v>24</v>
+        <v>21.55</v>
       </c>
       <c r="E25" s="2">
-        <v>4.58</v>
+        <v>5.3</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
-      <c r="K25" s="2">
-        <v>17.059999999999999</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="35"/>
-      <c r="B26" s="29" t="s">
-        <v>65</v>
-      </c>
+      <c r="K25" s="2"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="29"/>
+      <c r="B26" s="29"/>
       <c r="C26" s="2">
-        <v>-2.78</v>
+        <v>4.2300000000000004</v>
       </c>
       <c r="D26" s="2">
-        <v>21.55</v>
+        <v>29.3</v>
       </c>
       <c r="E26" s="2">
-        <v>5.3</v>
+        <v>3.78</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -1801,17 +1875,17 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="35"/>
-      <c r="B27" s="35"/>
+    <row r="27" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="29"/>
+      <c r="B27" s="29"/>
       <c r="C27" s="2">
-        <v>4.2300000000000004</v>
+        <v>1158.44</v>
       </c>
       <c r="D27" s="2">
-        <v>29.3</v>
+        <v>84.6</v>
       </c>
       <c r="E27" s="2">
-        <v>3.78</v>
+        <v>53.46</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -1820,17 +1894,17 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="35"/>
-      <c r="B28" s="35"/>
+    <row r="28" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="30"/>
+      <c r="B28" s="30"/>
       <c r="C28" s="2">
-        <v>1158.44</v>
+        <v>-1146.51</v>
       </c>
       <c r="D28" s="2">
-        <v>84.6</v>
+        <v>85.35</v>
       </c>
       <c r="E28" s="2">
-        <v>53.46</v>
+        <v>53.19</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1839,62 +1913,43 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="30"/>
-      <c r="B29" s="30"/>
+    <row r="29" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <v>75</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="C29" s="2">
-        <v>-1146.51</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="D29" s="2">
-        <v>85.35</v>
+        <v>9.82</v>
       </c>
       <c r="E29" s="2">
-        <v>53.19</v>
-      </c>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-    </row>
-    <row r="30" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="2">
-        <v>75</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C30" s="2">
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="D30" s="2">
-        <v>9.82</v>
-      </c>
-      <c r="E30" s="2">
         <v>66.64</v>
       </c>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A20:A24"/>
-    <mergeCell ref="B21:B24"/>
-    <mergeCell ref="A25:A29"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="A3:A8"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="A15:A19"/>
-    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="A19:A23"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="A24:A28"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B15:B18"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B11:B14"/>
-    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="B8:B9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1902,16 +1957,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D8BE7F8-7CAC-444A-9E19-C454CF5B63E1}">
-  <dimension ref="A2:K30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:K29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.21875" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="20.399999999999999" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A2" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>11</v>
@@ -1944,8 +1999,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="29">
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="28">
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1969,9 +2024,9 @@
         <v>28.2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="35"/>
-      <c r="B4" s="28" t="s">
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="29"/>
+      <c r="B4" s="32" t="s">
         <v>44</v>
       </c>
       <c r="C4" s="2">
@@ -1990,9 +2045,9 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="35"/>
-      <c r="B5" s="28"/>
+    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="29"/>
+      <c r="B5" s="32"/>
       <c r="C5" s="2">
         <v>40.93</v>
       </c>
@@ -2009,9 +2064,9 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="35"/>
-      <c r="B6" s="28"/>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="29"/>
+      <c r="B6" s="32"/>
       <c r="C6" s="2">
         <v>0.88</v>
       </c>
@@ -2028,9 +2083,9 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="30"/>
-      <c r="B7" s="28"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="2">
         <v>10</v>
       </c>
@@ -2047,12 +2102,12 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="29">
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="28">
         <v>0.05</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" s="2">
         <v>6.6</v>
@@ -2072,10 +2127,10 @@
         <v>29.4</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="35"/>
-      <c r="B9" s="28" t="s">
-        <v>58</v>
+    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="29"/>
+      <c r="B9" s="32" t="s">
+        <v>57</v>
       </c>
       <c r="C9" s="2">
         <v>36.79</v>
@@ -2093,9 +2148,9 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="35"/>
-      <c r="B10" s="28"/>
+    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="29"/>
+      <c r="B10" s="32"/>
       <c r="C10" s="2">
         <v>37.18</v>
       </c>
@@ -2112,9 +2167,9 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="35"/>
-      <c r="B11" s="28"/>
+    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="29"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="2">
         <v>0.87</v>
       </c>
@@ -2131,9 +2186,9 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="30"/>
-      <c r="B12" s="28"/>
+      <c r="B12" s="32"/>
       <c r="C12" s="2">
         <v>6</v>
       </c>
@@ -2150,8 +2205,8 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="29">
+    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="28">
         <v>0.1</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -2175,9 +2230,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="35"/>
-      <c r="B14" s="28" t="s">
+    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="29"/>
+      <c r="B14" s="32" t="s">
         <v>47</v>
       </c>
       <c r="C14" s="2">
@@ -2196,9 +2251,9 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="35"/>
-      <c r="B15" s="28"/>
+    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="29"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="2">
         <v>35.4</v>
       </c>
@@ -2215,9 +2270,9 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="35"/>
-      <c r="B16" s="28"/>
+    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="29"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="2">
         <v>0.87</v>
       </c>
@@ -2234,9 +2289,9 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="30"/>
-      <c r="B17" s="28"/>
+      <c r="B17" s="32"/>
       <c r="C17" s="2">
         <v>3</v>
       </c>
@@ -2253,8 +2308,8 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="29">
+    <row r="18" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="28">
         <v>0.2</v>
       </c>
       <c r="B18" s="2" t="s">
@@ -2278,9 +2333,9 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="35"/>
-      <c r="B19" s="28" t="s">
+    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="29"/>
+      <c r="B19" s="32" t="s">
         <v>47</v>
       </c>
       <c r="C19" s="2">
@@ -2299,9 +2354,9 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="35"/>
-      <c r="B20" s="28"/>
+    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="29"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="2">
         <v>33.1</v>
       </c>
@@ -2318,9 +2373,9 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="35"/>
-      <c r="B21" s="28"/>
+    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="29"/>
+      <c r="B21" s="32"/>
       <c r="C21" s="2">
         <v>1.2</v>
       </c>
@@ -2337,9 +2392,9 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="30"/>
-      <c r="B22" s="28"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="2">
         <v>3</v>
       </c>
@@ -2356,12 +2411,12 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="29">
+    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="28">
         <v>0.5</v>
       </c>
-      <c r="B23" s="29" t="s">
-        <v>59</v>
+      <c r="B23" s="28" t="s">
+        <v>58</v>
       </c>
       <c r="C23" s="2">
         <v>34.5</v>
@@ -2379,9 +2434,9 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="35"/>
-      <c r="B24" s="35"/>
+    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="29"/>
+      <c r="B24" s="29"/>
       <c r="C24" s="2">
         <v>18.899999999999999</v>
       </c>
@@ -2398,9 +2453,9 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="35"/>
-      <c r="B25" s="35"/>
+    <row r="25" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="29"/>
+      <c r="B25" s="29"/>
       <c r="C25" s="2">
         <v>0.56999999999999995</v>
       </c>
@@ -2417,7 +2472,7 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="30"/>
       <c r="B26" s="30"/>
       <c r="C26" s="2">
@@ -2436,11 +2491,11 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="29">
+    <row r="27" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="28">
         <v>0.7</v>
       </c>
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="28" t="s">
         <v>32</v>
       </c>
       <c r="C27" s="2">
@@ -2459,9 +2514,9 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="35"/>
-      <c r="B28" s="35"/>
+    <row r="28" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="29"/>
+      <c r="B28" s="29"/>
       <c r="C28" s="2">
         <v>13.8</v>
       </c>
@@ -2478,7 +2533,7 @@
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
     </row>
-    <row r="29" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="30"/>
       <c r="B29" s="30"/>
       <c r="C29" s="2">
@@ -2496,31 +2551,6 @@
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
-    </row>
-    <row r="30" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="2">
-        <v>1</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C30" s="2">
-        <v>28.2</v>
-      </c>
-      <c r="D30" s="2">
-        <v>10</v>
-      </c>
-      <c r="E30" s="2">
-        <v>84</v>
-      </c>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1">
-        <v>2.2999999999999998</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -2544,13 +2574,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF29AC17-26FE-4126-A8A6-4FFD9DE0E8DD}">
   <dimension ref="A2:K51"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.21875" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="20.399999999999999" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A2" s="7" t="s">
         <v>38</v>
       </c>
@@ -2585,8 +2615,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="33" t="s">
         <v>39</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -2610,9 +2640,9 @@
         <v>37.5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="26"/>
-      <c r="B4" s="28" t="s">
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="34"/>
+      <c r="B4" s="32" t="s">
         <v>44</v>
       </c>
       <c r="C4" s="2">
@@ -2631,9 +2661,9 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="26"/>
-      <c r="B5" s="28"/>
+    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="34"/>
+      <c r="B5" s="32"/>
       <c r="C5" s="2">
         <v>24.6</v>
       </c>
@@ -2650,9 +2680,9 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="26"/>
-      <c r="B6" s="28"/>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="34"/>
+      <c r="B6" s="32"/>
       <c r="C6" s="2">
         <v>34.4</v>
       </c>
@@ -2669,9 +2699,9 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="27"/>
-      <c r="B7" s="28"/>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="35"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="2">
         <v>0.99</v>
       </c>
@@ -2688,8 +2718,8 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="33" t="s">
         <v>40</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -2713,9 +2743,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="26"/>
-      <c r="B9" s="28" t="s">
+    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="34"/>
+      <c r="B9" s="32" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="2">
@@ -2734,9 +2764,9 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="26"/>
-      <c r="B10" s="28"/>
+    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="34"/>
+      <c r="B10" s="32"/>
       <c r="C10" s="2">
         <v>27.8</v>
       </c>
@@ -2753,9 +2783,9 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="27"/>
-      <c r="B11" s="28"/>
+    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="35"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="2">
         <v>0.85</v>
       </c>
@@ -2772,8 +2802,8 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="25" t="s">
+    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="33" t="s">
         <v>41</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -2797,9 +2827,9 @@
         <v>34.799999999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="26"/>
-      <c r="B13" s="28" t="s">
+    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="34"/>
+      <c r="B13" s="32" t="s">
         <v>46</v>
       </c>
       <c r="C13" s="2">
@@ -2818,9 +2848,9 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="26"/>
-      <c r="B14" s="28"/>
+    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="34"/>
+      <c r="B14" s="32"/>
       <c r="C14" s="2">
         <v>25.83</v>
       </c>
@@ -2837,9 +2867,9 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="27"/>
-      <c r="B15" s="28"/>
+    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="35"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="2">
         <v>0.85</v>
       </c>
@@ -2856,8 +2886,8 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
+    <row r="16" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="33" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="2" t="s">
@@ -2881,9 +2911,9 @@
         <v>33.799999999999997</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="26"/>
-      <c r="B17" s="28" t="s">
+    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="34"/>
+      <c r="B17" s="32" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="2">
@@ -2902,9 +2932,9 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="26"/>
-      <c r="B18" s="28"/>
+    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="34"/>
+      <c r="B18" s="32"/>
       <c r="C18" s="2">
         <v>25.83</v>
       </c>
@@ -2921,9 +2951,9 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="27"/>
-      <c r="B19" s="29"/>
+    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="35"/>
+      <c r="B19" s="28"/>
       <c r="C19" s="3">
         <v>0.85</v>
       </c>
@@ -2940,8 +2970,8 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="31" t="s">
+    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="36" t="s">
         <v>43</v>
       </c>
       <c r="B20" s="2" t="s">
@@ -2965,9 +2995,9 @@
         <v>28.5</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="31"/>
-      <c r="B21" s="28" t="s">
+    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="36"/>
+      <c r="B21" s="32" t="s">
         <v>47</v>
       </c>
       <c r="C21" s="2">
@@ -2986,9 +3016,9 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="31"/>
-      <c r="B22" s="28"/>
+    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="36"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="2">
         <v>17.5</v>
       </c>
@@ -3005,9 +3035,9 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="31"/>
-      <c r="B23" s="28"/>
+    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="36"/>
+      <c r="B23" s="32"/>
       <c r="C23" s="2">
         <v>41</v>
       </c>
@@ -3024,9 +3054,9 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="31"/>
-      <c r="B24" s="28"/>
+    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="36"/>
+      <c r="B24" s="32"/>
       <c r="C24" s="2">
         <v>1</v>
       </c>
@@ -3043,7 +3073,7 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
       <c r="B25" s="11"/>
       <c r="C25" s="10"/>
@@ -3056,7 +3086,7 @@
       <c r="J25" s="10"/>
       <c r="K25" s="10"/>
     </row>
-    <row r="26" spans="1:11" ht="21" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:11" ht="21.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26" s="12" t="s">
         <v>48</v>
       </c>
@@ -3091,8 +3121,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="32" t="s">
+    <row r="27" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="37" t="s">
         <v>39</v>
       </c>
       <c r="B27" s="15" t="s">
@@ -3116,13 +3146,13 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="33"/>
+    <row r="28" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="38"/>
       <c r="B28" s="6" t="s">
         <v>52</v>
       </c>
       <c r="C28" s="2">
-        <v>37</v>
+        <v>-37</v>
       </c>
       <c r="D28" s="2">
         <v>105.2</v>
@@ -3139,10 +3169,10 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="34"/>
+    <row r="29" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="39"/>
       <c r="B29" s="20" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C29" s="21">
         <v>32.299999999999997</v>
@@ -3162,8 +3192,8 @@
       <c r="J29" s="22"/>
       <c r="K29" s="23"/>
     </row>
-    <row r="30" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="26" t="s">
+    <row r="30" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="34" t="s">
         <v>40</v>
       </c>
       <c r="B30" s="4" t="s">
@@ -3187,9 +3217,9 @@
         <v>33.5</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="26"/>
-      <c r="B31" s="28" t="s">
+    <row r="31" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="34"/>
+      <c r="B31" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C31" s="2">
@@ -3208,9 +3238,9 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>
-    <row r="32" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="26"/>
-      <c r="B32" s="28"/>
+    <row r="32" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="34"/>
+      <c r="B32" s="32"/>
       <c r="C32" s="2">
         <v>38.9</v>
       </c>
@@ -3227,9 +3257,9 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
     </row>
-    <row r="33" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="26"/>
-      <c r="B33" s="28"/>
+    <row r="33" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="34"/>
+      <c r="B33" s="32"/>
       <c r="C33" s="2">
         <v>47.16</v>
       </c>
@@ -3246,9 +3276,9 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
     </row>
-    <row r="34" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="27"/>
-      <c r="B34" s="28"/>
+    <row r="34" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="35"/>
+      <c r="B34" s="32"/>
       <c r="C34" s="2">
         <v>0.96</v>
       </c>
@@ -3265,8 +3295,8 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
     </row>
-    <row r="35" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="25" t="s">
+    <row r="35" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="33" t="s">
         <v>41</v>
       </c>
       <c r="B35" s="2" t="s">
@@ -3290,9 +3320,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="26"/>
-      <c r="B36" s="28" t="s">
+    <row r="36" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="34"/>
+      <c r="B36" s="32" t="s">
         <v>10</v>
       </c>
       <c r="C36" s="2">
@@ -3311,9 +3341,9 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
     </row>
-    <row r="37" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="26"/>
-      <c r="B37" s="28"/>
+    <row r="37" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="34"/>
+      <c r="B37" s="32"/>
       <c r="C37" s="2">
         <v>13</v>
       </c>
@@ -3330,9 +3360,9 @@
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
     </row>
-    <row r="38" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="27"/>
-      <c r="B38" s="28"/>
+    <row r="38" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="35"/>
+      <c r="B38" s="32"/>
       <c r="C38" s="2">
         <v>35</v>
       </c>
@@ -3349,8 +3379,8 @@
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
     </row>
-    <row r="39" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="25" t="s">
+    <row r="39" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="33" t="s">
         <v>49</v>
       </c>
       <c r="B39" s="2" t="s">
@@ -3374,13 +3404,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="26"/>
+    <row r="40" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="34"/>
       <c r="B40" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C40" s="2">
-        <v>36.200000000000003</v>
+        <v>-36.200000000000003</v>
       </c>
       <c r="D40" s="2">
         <v>110</v>
@@ -3397,10 +3427,10 @@
         <v>74</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="27"/>
+    <row r="41" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="35"/>
       <c r="B41" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C41" s="2">
         <v>30.6</v>
@@ -3420,12 +3450,12 @@
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
     </row>
-    <row r="42" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="25" t="s">
+    <row r="42" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="33" t="s">
         <v>50</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C42" s="2">
         <v>15</v>
@@ -3443,10 +3473,10 @@
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
     </row>
-    <row r="43" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="26"/>
-      <c r="B43" s="28" t="s">
-        <v>63</v>
+    <row r="43" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A43" s="34"/>
+      <c r="B43" s="32" t="s">
+        <v>61</v>
       </c>
       <c r="C43" s="2">
         <v>33</v>
@@ -3464,9 +3494,9 @@
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
     </row>
-    <row r="44" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="26"/>
-      <c r="B44" s="28"/>
+    <row r="44" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A44" s="34"/>
+      <c r="B44" s="32"/>
       <c r="C44" s="2">
         <v>38.5</v>
       </c>
@@ -3483,9 +3513,9 @@
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
     </row>
-    <row r="45" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="26"/>
-      <c r="B45" s="28"/>
+    <row r="45" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A45" s="34"/>
+      <c r="B45" s="32"/>
       <c r="C45" s="2">
         <v>6</v>
       </c>
@@ -3502,9 +3532,9 @@
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
     </row>
-    <row r="46" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="27"/>
-      <c r="B46" s="28"/>
+    <row r="46" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A46" s="35"/>
+      <c r="B46" s="32"/>
       <c r="C46" s="2">
         <v>0.7</v>
       </c>
@@ -3521,12 +3551,12 @@
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
     </row>
-    <row r="47" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="25" t="s">
+    <row r="47" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="B47" s="29" t="s">
-        <v>68</v>
+      <c r="B47" s="28" t="s">
+        <v>65</v>
       </c>
       <c r="C47" s="2">
         <v>-973.2</v>
@@ -3544,8 +3574,8 @@
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
     </row>
-    <row r="48" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="26"/>
+    <row r="48" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A48" s="34"/>
       <c r="B48" s="30"/>
       <c r="C48" s="2">
         <v>1000.5</v>
@@ -3563,9 +3593,9 @@
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
     </row>
-    <row r="49" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="26"/>
-      <c r="B49" s="28" t="s">
+    <row r="49" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A49" s="34"/>
+      <c r="B49" s="32" t="s">
         <v>29</v>
       </c>
       <c r="C49" s="2">
@@ -3584,9 +3614,9 @@
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
     </row>
-    <row r="50" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="26"/>
-      <c r="B50" s="28"/>
+    <row r="50" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A50" s="34"/>
+      <c r="B50" s="32"/>
       <c r="C50" s="2">
         <v>34.1</v>
       </c>
@@ -3603,9 +3633,9 @@
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
     </row>
-    <row r="51" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A51" s="27"/>
-      <c r="B51" s="28"/>
+    <row r="51" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A51" s="35"/>
+      <c r="B51" s="32"/>
       <c r="C51" s="2">
         <v>1</v>
       </c>
@@ -3654,14 +3684,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C16C6F80-4315-44AF-A2E4-79655DC29A36}">
   <dimension ref="A2:K31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="31.2" x14ac:dyDescent="0.45">
-      <c r="A2" s="36" t="s">
+    <row r="2" spans="1:11" ht="31.5" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
         <v>36</v>
       </c>
       <c r="B2" s="8" t="s">
@@ -3695,7 +3725,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>50</v>
       </c>
@@ -3720,7 +3750,7 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>60</v>
       </c>
@@ -3745,8 +3775,8 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="29">
+    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="28">
         <v>70</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -3770,9 +3800,9 @@
         <v>34.799999999999997</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="35"/>
-      <c r="B6" s="28" t="s">
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="29"/>
+      <c r="B6" s="32" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="2">
@@ -3791,9 +3821,9 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="35"/>
-      <c r="B7" s="28"/>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="29"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="2">
         <v>25.83</v>
       </c>
@@ -3810,9 +3840,9 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="30"/>
-      <c r="B8" s="28"/>
+      <c r="B8" s="32"/>
       <c r="C8" s="2">
         <v>0.85</v>
       </c>
@@ -3829,8 +3859,8 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="29">
+    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="28">
         <v>80</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -3854,9 +3884,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="35"/>
-      <c r="B10" s="28" t="s">
+    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="29"/>
+      <c r="B10" s="32" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="2">
@@ -3875,9 +3905,9 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="35"/>
-      <c r="B11" s="28"/>
+    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="29"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="2">
         <v>28.55</v>
       </c>
@@ -3894,9 +3924,9 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="30"/>
-      <c r="B12" s="28"/>
+      <c r="B12" s="32"/>
       <c r="C12" s="2">
         <v>1.06</v>
       </c>
@@ -3913,8 +3943,8 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="29">
+    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="28">
         <v>90</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -3938,9 +3968,9 @@
         <v>24.2</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="35"/>
-      <c r="B14" s="28" t="s">
+    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="29"/>
+      <c r="B14" s="32" t="s">
         <v>29</v>
       </c>
       <c r="C14" s="2">
@@ -3959,9 +3989,9 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="35"/>
-      <c r="B15" s="28"/>
+    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="29"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="2">
         <v>32.6</v>
       </c>
@@ -3978,9 +4008,9 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="30"/>
-      <c r="B16" s="28"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="2">
         <v>0.87</v>
       </c>
@@ -3997,8 +4027,8 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="29">
+    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="28">
         <v>100</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -4022,9 +4052,9 @@
         <v>20.5</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="35"/>
-      <c r="B18" s="28" t="s">
+    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="29"/>
+      <c r="B18" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C18" s="2">
@@ -4043,9 +4073,9 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="35"/>
-      <c r="B19" s="28"/>
+    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="29"/>
+      <c r="B19" s="32"/>
       <c r="C19" s="2">
         <v>6.6</v>
       </c>
@@ -4062,9 +4092,9 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="35"/>
-      <c r="B20" s="28"/>
+    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="29"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="2">
         <v>35</v>
       </c>
@@ -4081,9 +4111,9 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="30"/>
-      <c r="B21" s="28"/>
+      <c r="B21" s="32"/>
       <c r="C21" s="2">
         <v>1</v>
       </c>
@@ -4100,8 +4130,8 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="28">
+    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="32">
         <v>110</v>
       </c>
       <c r="B22" s="2" t="s">
@@ -4125,9 +4155,9 @@
         <v>18.38</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="28"/>
-      <c r="B23" s="28" t="s">
+    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="32"/>
+      <c r="B23" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="2">
@@ -4146,9 +4176,9 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="28"/>
-      <c r="B24" s="28"/>
+    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="32"/>
+      <c r="B24" s="32"/>
       <c r="C24" s="2">
         <v>7.5</v>
       </c>
@@ -4165,9 +4195,9 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="28"/>
-      <c r="B25" s="28"/>
+    <row r="25" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="32"/>
+      <c r="B25" s="32"/>
       <c r="C25" s="2">
         <v>33.700000000000003</v>
       </c>
@@ -4184,9 +4214,9 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="28"/>
-      <c r="B26" s="28"/>
+    <row r="26" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="32"/>
+      <c r="B26" s="32"/>
       <c r="C26" s="2">
         <v>1</v>
       </c>
@@ -4203,8 +4233,8 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="28">
+    <row r="27" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="32">
         <v>120</v>
       </c>
       <c r="B27" s="2" t="s">
@@ -4228,9 +4258,9 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="28"/>
-      <c r="B28" s="28" t="s">
+    <row r="28" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="32"/>
+      <c r="B28" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C28" s="2">
@@ -4249,9 +4279,9 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="28"/>
-      <c r="B29" s="28"/>
+    <row r="29" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="32"/>
+      <c r="B29" s="32"/>
       <c r="C29" s="2">
         <v>6.9</v>
       </c>
@@ -4268,9 +4298,9 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
     </row>
-    <row r="30" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="28"/>
-      <c r="B30" s="28"/>
+    <row r="30" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="32"/>
+      <c r="B30" s="32"/>
       <c r="C30" s="2">
         <v>31.1</v>
       </c>
@@ -4287,9 +4317,9 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
     </row>
-    <row r="31" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="28"/>
-      <c r="B31" s="28"/>
+    <row r="31" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="32"/>
+      <c r="B31" s="32"/>
       <c r="C31" s="2">
         <v>1</v>
       </c>
@@ -4327,15 +4357,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E73309-2F42-4CCD-9BEE-92312AFAD90C}">
-  <dimension ref="A2:K27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:K28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.21875" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="33" x14ac:dyDescent="0.45">
-      <c r="A2" s="37" t="s">
+    <row r="2" spans="1:11" ht="33.75" x14ac:dyDescent="0.4">
+      <c r="A2" s="26" t="s">
         <v>37</v>
       </c>
       <c r="B2" s="8" t="s">
@@ -4369,8 +4399,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="28" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -4394,9 +4424,9 @@
         <v>8.3000000000000007</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="35"/>
-      <c r="B4" s="28" t="s">
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="29"/>
+      <c r="B4" s="32" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="2">
@@ -4415,9 +4445,9 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="35"/>
-      <c r="B5" s="28"/>
+    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="29"/>
+      <c r="B5" s="32"/>
       <c r="C5" s="2">
         <v>5</v>
       </c>
@@ -4434,9 +4464,9 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="30"/>
-      <c r="B6" s="28"/>
+      <c r="B6" s="32"/>
       <c r="C6" s="2">
         <v>0.7</v>
       </c>
@@ -4453,8 +4483,8 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="29" t="s">
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -4478,9 +4508,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="35"/>
-      <c r="B8" s="28" t="s">
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="29"/>
+      <c r="B8" s="32" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="2">
@@ -4499,9 +4529,9 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="35"/>
-      <c r="B9" s="28"/>
+    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="29"/>
+      <c r="B9" s="32"/>
       <c r="C9" s="2">
         <v>11.3</v>
       </c>
@@ -4518,9 +4548,9 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="30"/>
-      <c r="B10" s="28"/>
+      <c r="B10" s="32"/>
       <c r="C10" s="2">
         <v>0.8</v>
       </c>
@@ -4537,8 +4567,8 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="29" t="s">
+    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="28" t="s">
         <v>23</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -4562,10 +4592,10 @@
         <v>14.9</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="35"/>
-      <c r="B12" s="28" t="s">
-        <v>14</v>
+    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="29"/>
+      <c r="B12" s="32" t="s">
+        <v>68</v>
       </c>
       <c r="C12" s="2">
         <v>15.4</v>
@@ -4583,9 +4613,9 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="35"/>
-      <c r="B13" s="28"/>
+    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="29"/>
+      <c r="B13" s="32"/>
       <c r="C13" s="2">
         <v>22</v>
       </c>
@@ -4602,9 +4632,9 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="30"/>
-      <c r="B14" s="28"/>
+    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="29"/>
+      <c r="B14" s="32"/>
       <c r="C14" s="2">
         <v>20</v>
       </c>
@@ -4621,63 +4651,63 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>12</v>
-      </c>
+    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="30"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="2">
-        <v>6.2</v>
+        <v>0.82</v>
       </c>
       <c r="D15" s="2">
-        <v>3</v>
+        <v>175.45</v>
       </c>
       <c r="E15" s="2">
-        <v>2.9</v>
+        <v>7.82</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
-      <c r="K15" s="2">
-        <v>22.65</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="35"/>
-      <c r="B16" s="28" t="s">
-        <v>10</v>
+      <c r="K15" s="2"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="C16" s="2">
-        <v>29.5</v>
+        <v>6.2</v>
       </c>
       <c r="D16" s="2">
-        <v>35.54</v>
+        <v>3</v>
       </c>
       <c r="E16" s="2">
-        <v>41.04</v>
+        <v>2.9</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-    </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="35"/>
-      <c r="B17" s="28"/>
+      <c r="K16" s="2">
+        <v>22.65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="29"/>
+      <c r="B17" s="32" t="s">
+        <v>10</v>
+      </c>
       <c r="C17" s="2">
-        <v>24.05</v>
+        <v>29.5</v>
       </c>
       <c r="D17" s="2">
-        <v>87.47</v>
+        <v>35.54</v>
       </c>
       <c r="E17" s="2">
-        <v>20.67</v>
+        <v>41.04</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -4686,17 +4716,17 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="30"/>
-      <c r="B18" s="28"/>
+    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="29"/>
+      <c r="B18" s="32"/>
       <c r="C18" s="2">
-        <v>0.87</v>
+        <v>24.05</v>
       </c>
       <c r="D18" s="2">
-        <v>188.29</v>
+        <v>87.47</v>
       </c>
       <c r="E18" s="2">
-        <v>42.73</v>
+        <v>20.67</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -4705,63 +4735,63 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>15</v>
-      </c>
+    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="30"/>
+      <c r="B19" s="32"/>
       <c r="C19" s="2">
-        <v>7</v>
+        <v>0.87</v>
       </c>
       <c r="D19" s="2">
-        <v>4.2</v>
+        <v>188.29</v>
       </c>
       <c r="E19" s="2">
-        <v>8.9440000000000008</v>
+        <v>42.73</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
-      <c r="K19" s="2">
-        <v>34.9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="35"/>
-      <c r="B20" s="28" t="s">
-        <v>16</v>
+      <c r="K19" s="2"/>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="C20" s="2">
-        <v>40.380000000000003</v>
+        <v>7</v>
       </c>
       <c r="D20" s="2">
-        <v>26</v>
+        <v>4.2</v>
       </c>
       <c r="E20" s="2">
-        <v>31.4</v>
+        <v>8.9440000000000008</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-    </row>
-    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="35"/>
-      <c r="B21" s="28"/>
+      <c r="K20" s="2">
+        <v>34.9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="29"/>
+      <c r="B21" s="32" t="s">
+        <v>16</v>
+      </c>
       <c r="C21" s="2">
-        <v>25.83</v>
+        <v>40.380000000000003</v>
       </c>
       <c r="D21" s="2">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="E21" s="2">
-        <v>17.96</v>
+        <v>31.4</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -4770,17 +4800,17 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="30"/>
-      <c r="B22" s="28"/>
+    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="29"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="2">
-        <v>0.85</v>
+        <v>25.83</v>
       </c>
       <c r="D22" s="2">
-        <v>158</v>
+        <v>66</v>
       </c>
       <c r="E22" s="2">
-        <v>52.15</v>
+        <v>17.96</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -4789,65 +4819,65 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="30"/>
+      <c r="B23" s="32"/>
       <c r="C23" s="2">
-        <v>83</v>
+        <v>0.85</v>
       </c>
       <c r="D23" s="2">
-        <v>55</v>
+        <v>158</v>
       </c>
       <c r="E23" s="2">
-        <v>106</v>
+        <v>52.15</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
-      <c r="H23" s="2">
-        <v>6.1</v>
-      </c>
+      <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="29" t="s">
+    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" s="2">
+        <v>83</v>
+      </c>
+      <c r="D24" s="2">
+        <v>55</v>
+      </c>
+      <c r="E24" s="2">
+        <v>106</v>
+      </c>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2">
+        <v>6.1</v>
+      </c>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="29" t="s">
+      <c r="B25" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C25" s="2">
         <v>98</v>
-      </c>
-      <c r="D24" s="2">
-        <v>0</v>
-      </c>
-      <c r="E24" s="2">
-        <v>2.11</v>
-      </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
-    </row>
-    <row r="25" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="30"/>
-      <c r="B25" s="30"/>
-      <c r="C25" s="2">
-        <v>57</v>
       </c>
       <c r="D25" s="2">
         <v>0</v>
       </c>
       <c r="E25" s="2">
-        <v>2.2200000000000002</v>
+        <v>2.11</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
@@ -4856,70 +4886,89 @@
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
     </row>
-    <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="26" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="30"/>
+      <c r="B26" s="30"/>
       <c r="C26" s="2">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="D26" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26" s="2">
-        <v>26.4</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
-      <c r="H26" s="6">
-        <v>2.1</v>
-      </c>
+      <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
     </row>
-    <row r="27" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C27" s="2">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="D27" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" s="2">
-        <v>35</v>
+        <v>26.4</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="6">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
     </row>
+    <row r="28" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" s="2">
+        <v>36</v>
+      </c>
+      <c r="D28" s="2">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2">
+        <v>35</v>
+      </c>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A11:A15"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="B8:B10"/>
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="B4:B6"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="B21:B23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4928,13 +4977,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E9F8947-643C-49C6-AB36-BE8BA0D8FDD7}">
   <dimension ref="A2:K42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="20.399999999999999" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A2" s="7" t="s">
         <v>31</v>
       </c>
@@ -4969,7 +5018,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>10</v>
       </c>
@@ -4994,7 +5043,7 @@
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
     </row>
-    <row r="4" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>20</v>
       </c>
@@ -5019,7 +5068,7 @@
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
     </row>
-    <row r="5" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>30</v>
       </c>
@@ -5044,7 +5093,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
     </row>
-    <row r="6" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>40</v>
       </c>
@@ -5069,7 +5118,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
     </row>
-    <row r="7" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>50</v>
       </c>
@@ -5094,7 +5143,7 @@
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>60</v>
       </c>
@@ -5119,8 +5168,8 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="29">
+    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="28">
         <v>70</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -5144,9 +5193,9 @@
         <v>34.5</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="35"/>
-      <c r="B10" s="28" t="s">
+    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="29"/>
+      <c r="B10" s="32" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="2">
@@ -5165,9 +5214,9 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="35"/>
-      <c r="B11" s="28"/>
+    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="29"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="2">
         <v>40</v>
       </c>
@@ -5184,9 +5233,9 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="30"/>
-      <c r="B12" s="28"/>
+      <c r="B12" s="32"/>
       <c r="C12" s="2">
         <v>0.49</v>
       </c>
@@ -5203,8 +5252,8 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="29">
+    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="28">
         <v>80</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -5228,9 +5277,9 @@
         <v>34.799999999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="35"/>
-      <c r="B14" s="28" t="s">
+    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="29"/>
+      <c r="B14" s="32" t="s">
         <v>16</v>
       </c>
       <c r="C14" s="2">
@@ -5249,9 +5298,9 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="35"/>
-      <c r="B15" s="28"/>
+    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="29"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="2">
         <v>25.83</v>
       </c>
@@ -5268,9 +5317,9 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="30"/>
-      <c r="B16" s="28"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="2">
         <v>0.85</v>
       </c>
@@ -5287,8 +5336,8 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="29">
+    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="28">
         <v>90</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -5312,9 +5361,9 @@
         <v>35.200000000000003</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="35"/>
-      <c r="B18" s="28" t="s">
+    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="29"/>
+      <c r="B18" s="32" t="s">
         <v>10</v>
       </c>
       <c r="C18" s="2">
@@ -5333,9 +5382,9 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="35"/>
-      <c r="B19" s="28"/>
+    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="29"/>
+      <c r="B19" s="32"/>
       <c r="C19" s="2">
         <v>33.799999999999997</v>
       </c>
@@ -5352,9 +5401,9 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="30"/>
-      <c r="B20" s="28"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="2">
         <v>1</v>
       </c>
@@ -5371,8 +5420,8 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="29">
+    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="28">
         <v>100</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -5396,9 +5445,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="35"/>
-      <c r="B22" s="28" t="s">
+    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="29"/>
+      <c r="B22" s="32" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="2">
@@ -5417,9 +5466,9 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="35"/>
-      <c r="B23" s="28"/>
+    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="29"/>
+      <c r="B23" s="32"/>
       <c r="C23" s="2">
         <v>58.67</v>
       </c>
@@ -5436,9 +5485,9 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="30"/>
-      <c r="B24" s="28"/>
+      <c r="B24" s="32"/>
       <c r="C24" s="2">
         <v>1.0900000000000001</v>
       </c>
@@ -5455,8 +5504,8 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="28">
+    <row r="25" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="32">
         <v>110</v>
       </c>
       <c r="B25" s="2" t="s">
@@ -5480,9 +5529,9 @@
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="28"/>
-      <c r="B26" s="28" t="s">
+    <row r="26" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="32"/>
+      <c r="B26" s="32" t="s">
         <v>14</v>
       </c>
       <c r="C26" s="2">
@@ -5501,9 +5550,9 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="28"/>
-      <c r="B27" s="28"/>
+    <row r="27" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="32"/>
+      <c r="B27" s="32"/>
       <c r="C27" s="2">
         <v>64</v>
       </c>
@@ -5520,9 +5569,9 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="28"/>
-      <c r="B28" s="28"/>
+    <row r="28" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="32"/>
+      <c r="B28" s="32"/>
       <c r="C28" s="2">
         <v>1.0900000000000001</v>
       </c>
@@ -5539,8 +5588,8 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="28">
+    <row r="29" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="32">
         <v>120</v>
       </c>
       <c r="B29" s="2" t="s">
@@ -5564,9 +5613,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="28"/>
-      <c r="B30" s="28" t="s">
+    <row r="30" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="32"/>
+      <c r="B30" s="32" t="s">
         <v>14</v>
       </c>
       <c r="C30" s="2">
@@ -5585,9 +5634,9 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
     </row>
-    <row r="31" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="28"/>
-      <c r="B31" s="28"/>
+    <row r="31" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="32"/>
+      <c r="B31" s="32"/>
       <c r="C31" s="2">
         <v>12.5</v>
       </c>
@@ -5604,9 +5653,9 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>
-    <row r="32" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="28"/>
-      <c r="B32" s="28"/>
+    <row r="32" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="32"/>
+      <c r="B32" s="32"/>
       <c r="C32" s="2">
         <v>14</v>
       </c>
@@ -5623,8 +5672,8 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
     </row>
-    <row r="33" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="28">
+    <row r="33" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="32">
         <v>130</v>
       </c>
       <c r="B33" s="2" t="s">
@@ -5648,9 +5697,9 @@
         <v>37.5</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="28"/>
-      <c r="B34" s="28" t="s">
+    <row r="34" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="32"/>
+      <c r="B34" s="32" t="s">
         <v>34</v>
       </c>
       <c r="C34" s="2">
@@ -5669,9 +5718,9 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
     </row>
-    <row r="35" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="28"/>
-      <c r="B35" s="28"/>
+    <row r="35" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="32"/>
+      <c r="B35" s="32"/>
       <c r="C35" s="2">
         <v>2.0499999999999998</v>
       </c>
@@ -5688,9 +5737,9 @@
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
     </row>
-    <row r="36" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="28"/>
-      <c r="B36" s="28"/>
+    <row r="36" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="32"/>
+      <c r="B36" s="32"/>
       <c r="C36" s="2">
         <v>77.47</v>
       </c>
@@ -5707,11 +5756,11 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
     </row>
-    <row r="37" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="28">
+    <row r="37" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="32">
         <v>140</v>
       </c>
-      <c r="B37" s="28" t="s">
+      <c r="B37" s="32" t="s">
         <v>32</v>
       </c>
       <c r="C37" s="2">
@@ -5730,9 +5779,9 @@
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
     </row>
-    <row r="38" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="28"/>
-      <c r="B38" s="28"/>
+    <row r="38" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="32"/>
+      <c r="B38" s="32"/>
       <c r="C38" s="2">
         <v>78.8</v>
       </c>
@@ -5749,9 +5798,9 @@
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
     </row>
-    <row r="39" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="28"/>
-      <c r="B39" s="28"/>
+    <row r="39" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="32"/>
+      <c r="B39" s="32"/>
       <c r="C39" s="2">
         <v>26.77</v>
       </c>
@@ -5768,11 +5817,11 @@
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
     </row>
-    <row r="40" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="28">
+    <row r="40" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="32">
         <v>150</v>
       </c>
-      <c r="B40" s="28" t="s">
+      <c r="B40" s="32" t="s">
         <v>32</v>
       </c>
       <c r="C40" s="2">
@@ -5791,9 +5840,9 @@
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
     </row>
-    <row r="41" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="28"/>
-      <c r="B41" s="28"/>
+    <row r="41" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="32"/>
+      <c r="B41" s="32"/>
       <c r="C41" s="2">
         <v>85</v>
       </c>
@@ -5810,9 +5859,9 @@
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
     </row>
-    <row r="42" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="28"/>
-      <c r="B42" s="28"/>
+    <row r="42" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="32"/>
+      <c r="B42" s="32"/>
       <c r="C42" s="2">
         <v>43</v>
       </c>
@@ -5852,4 +5901,1051 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BEDF951-EDBD-4AB6-B638-AB5970498620}">
+  <dimension ref="A1:K50"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="29.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="31" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+    </row>
+    <row r="2" spans="1:11" ht="31.5" x14ac:dyDescent="0.4">
+      <c r="A2" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="28">
+        <v>50</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="27">
+        <v>0.53</v>
+      </c>
+      <c r="D3" s="27">
+        <v>-180.2</v>
+      </c>
+      <c r="E3" s="27">
+        <v>14.13</v>
+      </c>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+    </row>
+    <row r="4" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="29"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="27">
+        <v>6.5</v>
+      </c>
+      <c r="D4" s="27">
+        <v>-48.19</v>
+      </c>
+      <c r="E4" s="27">
+        <v>27.83</v>
+      </c>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="29"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="27">
+        <v>0.95</v>
+      </c>
+      <c r="D5" s="27">
+        <v>-95.94</v>
+      </c>
+      <c r="E5" s="27">
+        <v>12.17</v>
+      </c>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+    </row>
+    <row r="6" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A6" s="29"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="27">
+        <v>3.44</v>
+      </c>
+      <c r="D6" s="27">
+        <v>-38.82</v>
+      </c>
+      <c r="E6" s="27">
+        <v>67.27</v>
+      </c>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="30"/>
+      <c r="B7" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="2">
+        <v>20.47</v>
+      </c>
+      <c r="D7" s="2">
+        <v>877.71</v>
+      </c>
+      <c r="E7" s="2">
+        <v>285.81</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+    </row>
+    <row r="8" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A8" s="28">
+        <v>60</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="27">
+        <v>0.92</v>
+      </c>
+      <c r="D8" s="27">
+        <v>-171.13</v>
+      </c>
+      <c r="E8" s="27">
+        <v>15.27</v>
+      </c>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+    </row>
+    <row r="9" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A9" s="29"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="27">
+        <v>10.68</v>
+      </c>
+      <c r="D9" s="27">
+        <v>-81.03</v>
+      </c>
+      <c r="E9" s="27">
+        <v>29.68</v>
+      </c>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="27"/>
+    </row>
+    <row r="10" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A10" s="29"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="27">
+        <v>15.86</v>
+      </c>
+      <c r="D10" s="27">
+        <v>-28.76</v>
+      </c>
+      <c r="E10" s="27">
+        <v>27.41</v>
+      </c>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
+    </row>
+    <row r="11" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A11" s="29"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="27">
+        <v>1.25</v>
+      </c>
+      <c r="D11" s="27">
+        <v>54.76</v>
+      </c>
+      <c r="E11" s="27">
+        <v>26.78</v>
+      </c>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="30"/>
+      <c r="B12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="2">
+        <v>18.23</v>
+      </c>
+      <c r="D12" s="2">
+        <v>877.1</v>
+      </c>
+      <c r="E12" s="2">
+        <v>285.81</v>
+      </c>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+    </row>
+    <row r="13" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A13" s="28">
+        <v>70</v>
+      </c>
+      <c r="B13" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="27">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="D13" s="27">
+        <v>-70.66</v>
+      </c>
+      <c r="E13" s="27">
+        <v>35.31</v>
+      </c>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="27"/>
+    </row>
+    <row r="14" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A14" s="29"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="27">
+        <v>19.420000000000002</v>
+      </c>
+      <c r="D14" s="27">
+        <v>-17.71</v>
+      </c>
+      <c r="E14" s="27">
+        <v>22.26</v>
+      </c>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
+    </row>
+    <row r="15" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A15" s="29"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="27">
+        <v>1.66</v>
+      </c>
+      <c r="D15" s="27">
+        <v>-20.67</v>
+      </c>
+      <c r="E15" s="27">
+        <v>85.73</v>
+      </c>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="30"/>
+      <c r="B16" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1.08</v>
+      </c>
+      <c r="D16" s="2">
+        <v>187.3</v>
+      </c>
+      <c r="E16" s="2">
+        <v>59.51</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+    </row>
+    <row r="17" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A17" s="28">
+        <v>80</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="27">
+        <v>25.25</v>
+      </c>
+      <c r="D17" s="27">
+        <v>-13.9</v>
+      </c>
+      <c r="E17" s="27">
+        <v>20.22</v>
+      </c>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
+    </row>
+    <row r="18" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A18" s="29"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="27">
+        <v>22.98</v>
+      </c>
+      <c r="D18" s="27">
+        <v>-74.78</v>
+      </c>
+      <c r="E18" s="27">
+        <v>37.21</v>
+      </c>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+    </row>
+    <row r="19" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A19" s="29"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="27">
+        <v>4.49</v>
+      </c>
+      <c r="D19" s="27">
+        <v>6.6</v>
+      </c>
+      <c r="E19" s="27">
+        <v>11.2</v>
+      </c>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+    </row>
+    <row r="20" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A20" s="29"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="27">
+        <v>2.87</v>
+      </c>
+      <c r="D20" s="27">
+        <v>-12.22</v>
+      </c>
+      <c r="E20" s="27">
+        <v>51.07</v>
+      </c>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="30"/>
+      <c r="B21" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" s="2">
+        <v>1.08</v>
+      </c>
+      <c r="D21" s="2">
+        <v>189.94</v>
+      </c>
+      <c r="E21" s="2">
+        <v>59.54</v>
+      </c>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+    </row>
+    <row r="22" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A22" s="28">
+        <v>90</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="27">
+        <v>5.51</v>
+      </c>
+      <c r="D22" s="27">
+        <v>-120.21</v>
+      </c>
+      <c r="E22" s="27">
+        <v>15.82</v>
+      </c>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+    </row>
+    <row r="23" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A23" s="29"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="27">
+        <v>25.08</v>
+      </c>
+      <c r="D23" s="27">
+        <v>-69.209999999999994</v>
+      </c>
+      <c r="E23" s="27">
+        <v>36.869999999999997</v>
+      </c>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+    </row>
+    <row r="24" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A24" s="29"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="27">
+        <v>34.549999999999997</v>
+      </c>
+      <c r="D24" s="27">
+        <v>-3.58</v>
+      </c>
+      <c r="E24" s="27">
+        <v>20.329999999999998</v>
+      </c>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+    </row>
+    <row r="25" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A25" s="29"/>
+      <c r="B25" s="30"/>
+      <c r="C25" s="27">
+        <v>0.85</v>
+      </c>
+      <c r="D25" s="27">
+        <v>69.55</v>
+      </c>
+      <c r="E25" s="27">
+        <v>13.73</v>
+      </c>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="30"/>
+      <c r="B26" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" s="2">
+        <v>1.01</v>
+      </c>
+      <c r="D26" s="2">
+        <v>193.82</v>
+      </c>
+      <c r="E26" s="2">
+        <v>64.12</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+    </row>
+    <row r="27" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A27" s="28">
+        <v>100</v>
+      </c>
+      <c r="B27" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="27">
+        <v>0.99</v>
+      </c>
+      <c r="D27" s="27">
+        <v>-177.55</v>
+      </c>
+      <c r="E27" s="27">
+        <v>5.78</v>
+      </c>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="27"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
+    </row>
+    <row r="28" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A28" s="29"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="27">
+        <v>11.35</v>
+      </c>
+      <c r="D28" s="27">
+        <v>-115.06</v>
+      </c>
+      <c r="E28" s="27">
+        <v>21.83</v>
+      </c>
+      <c r="F28" s="27"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="27"/>
+      <c r="K28" s="27"/>
+    </row>
+    <row r="29" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A29" s="29"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="27">
+        <v>23.57</v>
+      </c>
+      <c r="D29" s="27">
+        <v>-57.63</v>
+      </c>
+      <c r="E29" s="27">
+        <v>36.5</v>
+      </c>
+      <c r="F29" s="27"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="27"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="27"/>
+    </row>
+    <row r="30" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A30" s="29"/>
+      <c r="B30" s="30"/>
+      <c r="C30" s="27">
+        <v>21.34</v>
+      </c>
+      <c r="D30" s="27">
+        <v>-33.770000000000003</v>
+      </c>
+      <c r="E30" s="27">
+        <v>1.58</v>
+      </c>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="27"/>
+      <c r="J30" s="27"/>
+      <c r="K30" s="27"/>
+    </row>
+    <row r="31" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A31" s="29"/>
+      <c r="B31" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" s="27">
+        <v>24.11</v>
+      </c>
+      <c r="D31" s="27">
+        <v>9.58</v>
+      </c>
+      <c r="E31" s="27">
+        <v>15.53</v>
+      </c>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="27"/>
+      <c r="J31" s="27"/>
+      <c r="K31" s="27"/>
+    </row>
+    <row r="32" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A32" s="29"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="27">
+        <v>26.97</v>
+      </c>
+      <c r="D32" s="27">
+        <v>-19.170000000000002</v>
+      </c>
+      <c r="E32" s="27">
+        <v>25.94</v>
+      </c>
+      <c r="F32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="27"/>
+      <c r="J32" s="27"/>
+      <c r="K32" s="27"/>
+    </row>
+    <row r="33" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A33" s="29"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="27">
+        <v>0.83</v>
+      </c>
+      <c r="D33" s="27">
+        <v>64.67</v>
+      </c>
+      <c r="E33" s="27">
+        <v>12.37</v>
+      </c>
+      <c r="F33" s="27"/>
+      <c r="G33" s="27"/>
+      <c r="H33" s="27"/>
+      <c r="I33" s="27"/>
+      <c r="J33" s="27"/>
+      <c r="K33" s="27"/>
+    </row>
+    <row r="34" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="30"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="2">
+        <v>1.07</v>
+      </c>
+      <c r="D34" s="2">
+        <v>-182.6</v>
+      </c>
+      <c r="E34" s="2">
+        <v>49.16</v>
+      </c>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+    </row>
+    <row r="35" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A35" s="28">
+        <v>110</v>
+      </c>
+      <c r="B35" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="C35" s="27">
+        <v>0.82</v>
+      </c>
+      <c r="D35" s="27">
+        <v>-176.56</v>
+      </c>
+      <c r="E35" s="27">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="F35" s="27"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="27"/>
+      <c r="I35" s="27"/>
+      <c r="J35" s="27"/>
+      <c r="K35" s="27"/>
+    </row>
+    <row r="36" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A36" s="29"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="27">
+        <v>11.55</v>
+      </c>
+      <c r="D36" s="27">
+        <v>-118.22</v>
+      </c>
+      <c r="E36" s="27">
+        <v>17.75</v>
+      </c>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27"/>
+      <c r="I36" s="27"/>
+      <c r="J36" s="27"/>
+      <c r="K36" s="27"/>
+    </row>
+    <row r="37" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A37" s="29"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="27">
+        <v>2.59</v>
+      </c>
+      <c r="D37" s="27">
+        <v>-92.23</v>
+      </c>
+      <c r="E37" s="27">
+        <v>9.6300000000000008</v>
+      </c>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="27"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="27"/>
+    </row>
+    <row r="38" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A38" s="29"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="27">
+        <v>23.04</v>
+      </c>
+      <c r="D38" s="27">
+        <v>-57.67</v>
+      </c>
+      <c r="E38" s="27">
+        <v>35.21</v>
+      </c>
+      <c r="F38" s="27"/>
+      <c r="G38" s="27"/>
+      <c r="H38" s="27"/>
+      <c r="I38" s="27"/>
+      <c r="J38" s="27"/>
+      <c r="K38" s="27"/>
+    </row>
+    <row r="39" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A39" s="29"/>
+      <c r="B39" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="27">
+        <v>24.3</v>
+      </c>
+      <c r="D39" s="27">
+        <v>15.99</v>
+      </c>
+      <c r="E39" s="27">
+        <v>13.55</v>
+      </c>
+      <c r="F39" s="27"/>
+      <c r="G39" s="27"/>
+      <c r="H39" s="27"/>
+      <c r="I39" s="27"/>
+      <c r="J39" s="27"/>
+      <c r="K39" s="27"/>
+    </row>
+    <row r="40" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A40" s="29"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="27">
+        <v>28.29</v>
+      </c>
+      <c r="D40" s="27">
+        <v>-10.17</v>
+      </c>
+      <c r="E40" s="27">
+        <v>22.68</v>
+      </c>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="27"/>
+      <c r="I40" s="27"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="27"/>
+    </row>
+    <row r="41" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A41" s="29"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="27">
+        <v>0.78</v>
+      </c>
+      <c r="D41" s="27">
+        <v>66.47</v>
+      </c>
+      <c r="E41" s="27">
+        <v>11</v>
+      </c>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="27"/>
+      <c r="I41" s="27"/>
+      <c r="J41" s="27"/>
+      <c r="K41" s="27"/>
+    </row>
+    <row r="42" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="30"/>
+      <c r="B42" s="30"/>
+      <c r="C42" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="D42" s="2">
+        <v>174.81</v>
+      </c>
+      <c r="E42" s="2">
+        <v>45.57</v>
+      </c>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+    </row>
+    <row r="43" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A43" s="28">
+        <v>120</v>
+      </c>
+      <c r="B43" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C43" s="27">
+        <v>0.96</v>
+      </c>
+      <c r="D43" s="27">
+        <v>-173.81</v>
+      </c>
+      <c r="E43" s="27">
+        <v>7.63</v>
+      </c>
+      <c r="F43" s="27"/>
+      <c r="G43" s="27"/>
+      <c r="H43" s="27"/>
+      <c r="I43" s="27"/>
+      <c r="J43" s="27"/>
+      <c r="K43" s="27"/>
+    </row>
+    <row r="44" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A44" s="29"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="27">
+        <v>7.14</v>
+      </c>
+      <c r="D44" s="27">
+        <v>-120.04</v>
+      </c>
+      <c r="E44" s="27">
+        <v>17.52</v>
+      </c>
+      <c r="F44" s="27"/>
+      <c r="G44" s="27"/>
+      <c r="H44" s="27"/>
+      <c r="I44" s="27"/>
+      <c r="J44" s="27"/>
+      <c r="K44" s="27"/>
+    </row>
+    <row r="45" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A45" s="29"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="27">
+        <v>16.63</v>
+      </c>
+      <c r="D45" s="27">
+        <v>-91.35</v>
+      </c>
+      <c r="E45" s="27">
+        <v>23.08</v>
+      </c>
+      <c r="F45" s="27"/>
+      <c r="G45" s="27"/>
+      <c r="H45" s="27"/>
+      <c r="I45" s="27"/>
+      <c r="J45" s="27"/>
+      <c r="K45" s="27"/>
+    </row>
+    <row r="46" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A46" s="29"/>
+      <c r="B46" s="30"/>
+      <c r="C46" s="27">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="D46" s="27">
+        <v>-45.58</v>
+      </c>
+      <c r="E46" s="27">
+        <v>21.21</v>
+      </c>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27"/>
+      <c r="H46" s="27"/>
+      <c r="I46" s="27"/>
+      <c r="J46" s="27"/>
+      <c r="K46" s="27"/>
+    </row>
+    <row r="47" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A47" s="29"/>
+      <c r="B47" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="C47" s="27">
+        <v>34.270000000000003</v>
+      </c>
+      <c r="D47" s="27">
+        <v>18.440000000000001</v>
+      </c>
+      <c r="E47" s="27">
+        <v>14.01</v>
+      </c>
+      <c r="F47" s="27"/>
+      <c r="G47" s="27"/>
+      <c r="H47" s="27"/>
+      <c r="I47" s="27"/>
+      <c r="J47" s="27"/>
+      <c r="K47" s="27"/>
+    </row>
+    <row r="48" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A48" s="29"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="27">
+        <v>23.25</v>
+      </c>
+      <c r="D48" s="27">
+        <v>-13.18</v>
+      </c>
+      <c r="E48" s="27">
+        <v>17.829999999999998</v>
+      </c>
+      <c r="F48" s="27"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="27"/>
+      <c r="I48" s="27"/>
+      <c r="J48" s="27"/>
+      <c r="K48" s="27"/>
+    </row>
+    <row r="49" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A49" s="29"/>
+      <c r="B49" s="29"/>
+      <c r="C49" s="27">
+        <v>0.74</v>
+      </c>
+      <c r="D49" s="27">
+        <v>65.569999999999993</v>
+      </c>
+      <c r="E49" s="27">
+        <v>9.5299999999999994</v>
+      </c>
+      <c r="F49" s="27"/>
+      <c r="G49" s="27"/>
+      <c r="H49" s="27"/>
+      <c r="I49" s="27"/>
+      <c r="J49" s="27"/>
+      <c r="K49" s="27"/>
+    </row>
+    <row r="50" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A50" s="30"/>
+      <c r="B50" s="30"/>
+      <c r="C50" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="D50" s="2">
+        <v>171.14</v>
+      </c>
+      <c r="E50" s="2">
+        <v>48.99</v>
+      </c>
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
+      <c r="J50" s="2"/>
+      <c r="K50" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="A22:A26"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="A27:A34"/>
+    <mergeCell ref="B31:B34"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B6"/>
+    <mergeCell ref="A35:A42"/>
+    <mergeCell ref="B35:B38"/>
+    <mergeCell ref="B39:B42"/>
+    <mergeCell ref="A43:A50"/>
+    <mergeCell ref="B43:B46"/>
+    <mergeCell ref="B47:B50"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>